<commit_message>
Add UCloud (688158), Eoptolink (300502), Innolight (300308) and VNET US
Per request: add UCloud Technology (688158.SS, STAR cloud/AI compute),
Eoptolink (300502.SZ, optical modules) plus peer Zhongji Innolight
(300308.SZ, world #1 optical transceiver maker), and VNET Group's US ADR
(Nasdaq) under a dedicated 'US ADR (China)' group. 46 names total.

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/semi_datacenter_coverage.xlsx
+++ b/semi_datacenter_coverage.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -520,7 +520,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of 2026-07-08. Scope: mainland China, Hong Kong, Taiwan, South Korea, Japan, Singapore, Malaysia listings only - no US or Europe listings. Market caps approximate/rounded for scoping only (not investment advice). Recent IPOs/listings highlighted in green.</t>
+          <t>As of 2026-07-08. Scope: mainland China, Hong Kong, Taiwan, South Korea, Japan, Singapore, Malaysia listings, plus VNET (US-listed China ADR). Market caps approximate/rounded for scoping only (not investment advice). Recent IPOs/listings highlighted in green.</t>
         </is>
       </c>
     </row>
@@ -626,22 +626,22 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>SMIC</t>
+          <t>Zhongji Innolight</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>688981.SS / 0981.HK</t>
+          <t>300308.SZ</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>SSE STAR / HKEX</t>
+          <t>SZSE ChiNext</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Semis - Foundry</t>
+          <t>Data Center - Optical Modules</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
@@ -659,34 +659,34 @@
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>2020-07 (STAR) / 2004-03 (HK)</t>
+          <t>2012-04 (Innolight inj. 2017)</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr">
         <is>
-          <t>China's largest foundry; advanced-node localization flagship amid export controls.</t>
+          <t>World #1 optical transceiver maker (800G/1.6T); NVIDIA/hyperscaler supplier; HK listing filed.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Cambricon Technologies</t>
+          <t>SMIC</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>688256.SS</t>
+          <t>688981.SS / 0981.HK</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>SSE STAR</t>
+          <t>SSE STAR / HKEX</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Semis - AI Accelerators</t>
+          <t>Semis - Foundry</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -704,24 +704,24 @@
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>2020-07</t>
+          <t>2020-07 (STAR) / 2004-03 (HK)</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>China AI training/inference chip champion; revenue up &gt;4,000% YoY in 1H25; NVIDIA substitution play.</t>
+          <t>China's largest foundry; advanced-node localization flagship amid export controls.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Hygon Information Technology</t>
+          <t>Cambricon Technologies</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>688041.SS</t>
+          <t>688256.SS</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Semis - CPU/DCU</t>
+          <t>Semis - AI Accelerators</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -740,7 +740,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
@@ -749,34 +749,34 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>2022-08</t>
+          <t>2020-07</t>
         </is>
       </c>
       <c r="I9" s="10" t="inlineStr">
         <is>
-          <t>Domestic x86-compatible server CPUs + DCU accelerators; merging with Sugon (server OEM).</t>
+          <t>China AI training/inference chip champion; revenue up &gt;4,000% YoY in 1H25; NVIDIA substitution play.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>NAURA Technology</t>
+          <t>Hygon Information Technology</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>002371.SZ</t>
+          <t>688041.SS</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>SZSE</t>
+          <t>SSE STAR</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Semis - Equipment (WFE)</t>
+          <t>Semis - CPU/DCU</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
@@ -794,204 +794,204 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>2010-06</t>
+          <t>2022-08</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr">
         <is>
-          <t>China's largest domestic WFE maker; etch/deposition/thermal; localization play.</t>
+          <t>Domestic x86-compatible server CPUs + DCU accelerators; merging with Sugon (server OEM).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Moore Threads</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>688795.SS</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>SSE STAR</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Semis - GPU</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Eoptolink Technology</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>300502.SZ</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>SZSE ChiNext</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Data Center - Optical Modules</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Mainland China</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
-        <v>43</v>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>'China's NVIDIA'; full-function GPUs (MUSA architecture); raised ~$1.1B, +400% on debut.</t>
+      <c r="F11" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>2016-03</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>China #2 optical module maker (800G/1.6T); FY25 net profit +236%; planning HK H-share listing.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
+          <t>NAURA Technology</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>002371.SZ</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>SZSE</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Semis - Equipment (WFE)</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Mainland China</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>2010-06</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>China's largest domestic WFE maker; etch/deposition/thermal; localization play.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Moore Threads</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>688795.SS</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>SSE STAR</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Semis - GPU</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Mainland China</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>'China's NVIDIA'; full-function GPUs (MUSA architecture); raised ~$1.1B, +400% on debut.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
           <t>Hua Hong Semiconductor</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>688347.SS / 1347.HK</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>SSE STAR / HKEX</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Semis - Foundry</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Mainland China</t>
         </is>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="F14" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>2023-08 (STAR) / 2014-10 (HK)</t>
         </is>
       </c>
-      <c r="I12" s="10" t="inlineStr">
+      <c r="I14" s="10" t="inlineStr">
         <is>
           <t>China #2 foundry; specialty/mature nodes; power &amp; analog platforms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>AMEC (Advanced Micro-Fabrication)</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>688012.SS</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>SSE STAR</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Semis - Equipment (WFE)</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Mainland China</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>2019-07</t>
-        </is>
-      </c>
-      <c r="I13" s="10" t="inlineStr">
-        <is>
-          <t>China etch equipment leader; MOCVD; leading-edge localization.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>MetaX Integrated Circuits</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>688802.SS</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>SSE STAR</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Semis - GPU</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Mainland China</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="inlineStr">
-        <is>
-          <t>Domestic GPU for AI training/inference (Xiyun C500); founded by ex-AMD execs; ~700% debut pop.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Montage Technology</t>
+          <t>AMEC (Advanced Micro-Fabrication)</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>688008.SS</t>
+          <t>688012.SS</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Semis - Memory Interface</t>
+          <t>Semis - Equipment (WFE)</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="F15" s="9" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
@@ -1024,74 +1024,74 @@
       </c>
       <c r="I15" s="10" t="inlineStr">
         <is>
-          <t>DDR5 memory interface / CXL chips for servers; AI memory bandwidth beneficiary.</t>
+          <t>China etch equipment leader; MOCVD; leading-edge localization.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>GigaDevice Semiconductor</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>603986.SS</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>SSE</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Semis - Memory (NOR/NAND/DRAM)</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>MetaX Integrated Circuits</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>688802.SS</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>SSE STAR</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Semis - GPU</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Mainland China</t>
         </is>
       </c>
-      <c r="F16" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>2016-08</t>
-        </is>
-      </c>
-      <c r="I16" s="10" t="inlineStr">
-        <is>
-          <t>NOR flash leader; expanding niche DRAM (CXMT ecosystem partner); MCUs.</t>
+      <c r="F16" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Domestic GPU for AI training/inference (Xiyun C500); founded by ex-AMD execs; ~700% debut pop.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Runze Technology</t>
+          <t>Montage Technology</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>300442.SZ</t>
+          <t>688008.SS</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>SZSE ChiNext</t>
+          <t>SSE STAR</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Data Center - Wholesale IDC</t>
+          <t>Semis - Memory Interface</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="F17" s="9" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
@@ -1109,34 +1109,34 @@
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>2015 (backdoor 2022)</t>
+          <t>2019-07</t>
         </is>
       </c>
       <c r="I17" s="10" t="inlineStr">
         <is>
-          <t>Pure-play wholesale IDC campuses (Beijing-Langfang, Yangtze Delta); AI/intelligent-computing demand.</t>
+          <t>DDR5 memory interface / CXL chips for servers; AI memory bandwidth beneficiary.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Beijing Sinnet Technology</t>
+          <t>GigaDevice Semiconductor</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>300383.SZ</t>
+          <t>603986.SS</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>SZSE ChiNext</t>
+          <t>SSE</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Data Center - IDC/Cloud</t>
+          <t>Semis - Memory (NOR/NAND/DRAM)</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="F18" s="9" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
@@ -1154,140 +1154,178 @@
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>2014-01</t>
+          <t>2016-08</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
-          <t>Beijing-area IDC + AWS China (Ningxia/Beijing) cloud operator.</t>
+          <t>NOR flash leader; expanding niche DRAM (CXMT ecosystem partner); MCUs.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
+          <t>Runze Technology</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>300442.SZ</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>SZSE ChiNext</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Data Center - Wholesale IDC</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Mainland China</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>2015 (backdoor 2022)</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>Pure-play wholesale IDC campuses (Beijing-Langfang, Yangtze Delta); AI/intelligent-computing demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Beijing Sinnet Technology</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>300383.SZ</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>SZSE ChiNext</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Data Center - IDC/Cloud</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Mainland China</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>2014-01</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>Beijing-area IDC + AWS China (Ningxia/Beijing) cloud operator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
           <t>Shanghai AtHub</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>603881.SS</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>SSE</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>Data Center - Wholesale IDC</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Mainland China</t>
         </is>
       </c>
-      <c r="F19" s="9" t="n">
+      <c r="F21" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
         <is>
           <t>2017-01</t>
         </is>
       </c>
-      <c r="I19" s="10" t="inlineStr">
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>Wholesale datacenter developer; anchor customer Alibaba; East China AI capacity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>HONG KONG</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Biren Technology</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>6082.HK</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>HKEX</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Semis - GPU</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Hong Kong</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="I21" s="7" t="inlineStr">
-        <is>
-          <t>High-performance GPU designer (BR20X/BR30X); raised ~$717M in Jan-2026 HK IPO, +76% debut.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>ASMPT</t>
+          <t>UCloud Technology</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>0522.HK</t>
+          <t>688158.SS</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>HKEX</t>
+          <t>SSE STAR</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Semis - Equipment (Packaging)</t>
+          <t>Data Center - Cloud/AI Compute</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Mainland China</t>
         </is>
       </c>
       <c r="F22" s="9" t="n">
-        <v>11</v>
+        <v>2.3</v>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
@@ -1296,69 +1334,31 @@
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>1989-06</t>
+          <t>2020-01</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
-          <t>Advanced packaging equipment leader; TCB bonders for HBM/CoWoS; key AI memory enabler.</t>
+          <t>Neutral third-party cloud provider; Kongming AI compute platform; first cloud company listed on STAR.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Horizon Robotics</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>9660.HK</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>HKEX</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Semis - Auto AI SoC</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Hong Kong</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>2024-10</t>
-        </is>
-      </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>Leading China ADAS/AD computing SoC (Journey series); largest HK tech IPO of 2024.</t>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>HONG KONG</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>InnoScience</t>
+          <t>Biren Technology</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>2577.HK</t>
+          <t>6082.HK</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Semis - Power (GaN)</t>
+          <t>Semis - GPU</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1377,7 +1377,7 @@
         </is>
       </c>
       <c r="F24" s="6" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
@@ -1386,34 +1386,34 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>World's largest GaN-on-Si IDM; AI server power / fast-charging adoption.</t>
+          <t>High-performance GPU designer (BR20X/BR30X); raised ~$717M in Jan-2026 HK IPO, +76% debut.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>GDS Holdings</t>
+          <t>ASMPT</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>9698.HK (also GDS US ADR)</t>
+          <t>0522.HK</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>HKEX (dual-primary)</t>
+          <t>HKEX</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Data Center - Colocation</t>
+          <t>Semis - Equipment (Packaging)</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -1422,7 +1422,7 @@
         </is>
       </c>
       <c r="F25" s="9" t="n">
-        <v>6.7</v>
+        <v>11</v>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
@@ -1431,69 +1431,69 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>2022-01 (HK) / 2016-11 (ADR)</t>
+          <t>1989-06</t>
         </is>
       </c>
       <c r="I25" s="10" t="inlineStr">
         <is>
-          <t>Carrier-neutral hyperscale colo leader in China; AI-driven wholesale demand; DayOne (international) angle.</t>
+          <t>Advanced packaging equipment leader; TCB bonders for HBM/CoWoS; key AI memory enabler.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>SUNeVision Holdings</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>1686.HK</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Horizon Robotics</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>9660.HK</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>HKEX</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Data Center - Colocation</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Semis - Auto AI SoC</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="F26" s="9" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H26" s="8" t="inlineStr">
-        <is>
-          <t>2000-03</t>
-        </is>
-      </c>
-      <c r="I26" s="10" t="inlineStr">
-        <is>
-          <t>Hong Kong's largest carrier-neutral datacenter operator (iAdvantage); SHKP-backed; MEGA campuses.</t>
+      <c r="F26" s="6" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>Leading China ADAS/AD computing SoC (Journey series); largest HK tech IPO of 2024.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Black Sesame International</t>
+          <t>InnoScience</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2533.HK</t>
+          <t>2577.HK</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Semis - Auto AI SoC</t>
+          <t>Semis - Power (GaN)</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="F27" s="6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
@@ -1521,50 +1521,88 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>Auto-grade AI SoCs (Huashan/Wudang); first 18C-chapter HK listing.</t>
+          <t>World's largest GaN-on-Si IDM; AI server power / fast-charging adoption.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>TAIWAN</t>
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>GDS Holdings</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>9698.HK (also GDS US ADR)</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>HKEX (dual-primary)</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Data Center - Colocation</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>2022-01 (HK) / 2016-11 (ADR)</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t>Carrier-neutral hyperscale colo leader in China; AI-driven wholesale demand; DayOne (international) angle.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>SUNeVision Holdings</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>2330.TW</t>
+          <t>1686.HK</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>TWSE</t>
+          <t>HKEX</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Semis - Foundry</t>
+          <t>Data Center - Colocation</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="F29" s="9" t="n">
-        <v>1200</v>
+        <v>2.7</v>
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
@@ -1573,114 +1611,76 @@
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>1994-09</t>
+          <t>2000-03</t>
         </is>
       </c>
       <c r="I29" s="10" t="inlineStr">
         <is>
-          <t>World's leading-edge foundry; CoWoS/advanced packaging bottleneck for AI accelerators.</t>
+          <t>Hong Kong's largest carrier-neutral datacenter operator (iAdvantage); SHKP-backed; MEGA campuses.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>Hon Hai Precision (Foxconn)</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>2317.TW</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>TWSE</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Data Center - AI Servers (ODM)</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="n">
-        <v>100</v>
-      </c>
-      <c r="G30" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H30" s="8" t="inlineStr">
-        <is>
-          <t>1991-06</t>
-        </is>
-      </c>
-      <c r="I30" s="10" t="inlineStr">
-        <is>
-          <t>Largest AI server assembler (GB200/GB300 racks); NVIDIA's key systems partner.</t>
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Black Sesame International</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>2533.HK</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>HKEX</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Semis - Auto AI SoC</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>Auto-grade AI SoCs (Huashan/Wudang); first 18C-chapter HK listing.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>MediaTek</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>2454.TW</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>TWSE</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Semis - Fabless (SoC)</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H31" s="8" t="inlineStr">
-        <is>
-          <t>2001-07</t>
-        </is>
-      </c>
-      <c r="I31" s="10" t="inlineStr">
-        <is>
-          <t>Mobile/connectivity SoC leader; custom ASIC push into AI datacenter (with Google/others).</t>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>TAIWAN</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>Delta Electronics</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>2308.TW</t>
+          <t>2330.TW</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Data Center - Power/Cooling</t>
+          <t>Semis - Foundry</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="F32" s="9" t="n">
-        <v>60</v>
+        <v>1200</v>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
@@ -1708,24 +1708,24 @@
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>1988-12</t>
+          <t>1994-09</t>
         </is>
       </c>
       <c r="I32" s="10" t="inlineStr">
         <is>
-          <t>Datacenter power supplies, busbars, liquid cooling; key AI rack power beneficiary.</t>
+          <t>World's leading-edge foundry; CoWoS/advanced packaging bottleneck for AI accelerators.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Quanta Computer</t>
+          <t>Hon Hai Precision (Foxconn)</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>2382.TW</t>
+          <t>2317.TW</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
@@ -1744,7 +1744,7 @@
         </is>
       </c>
       <c r="F33" s="9" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
@@ -1753,24 +1753,24 @@
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>1999-01</t>
+          <t>1991-06</t>
         </is>
       </c>
       <c r="I33" s="10" t="inlineStr">
         <is>
-          <t>Top AI server ODM for US hyperscalers; cloud infrastructure leverage.</t>
+          <t>Largest AI server assembler (GB200/GB300 racks); NVIDIA's key systems partner.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>Wiwynn</t>
+          <t>MediaTek</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>6669.TW</t>
+          <t>2454.TW</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Data Center - AI Servers (ODM)</t>
+          <t>Semis - Fabless (SoC)</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="F34" s="9" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
@@ -1798,24 +1798,24 @@
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>2019-03</t>
+          <t>2001-07</t>
         </is>
       </c>
       <c r="I34" s="10" t="inlineStr">
         <is>
-          <t>Hyperscale-focused server pure-play (Wistron spin-off); Meta/Microsoft exposure.</t>
+          <t>Mobile/connectivity SoC leader; custom ASIC push into AI datacenter (with Google/others).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>ASE Technology Holding</t>
+          <t>Delta Electronics</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>3711.TW</t>
+          <t>2308.TW</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Semis - OSAT</t>
+          <t>Data Center - Power/Cooling</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="F35" s="9" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
@@ -1843,24 +1843,24 @@
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>2018-04 (holding)</t>
+          <t>1988-12</t>
         </is>
       </c>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>World's largest OSAT; advanced packaging/test capacity for AI chips.</t>
+          <t>Datacenter power supplies, busbars, liquid cooling; key AI rack power beneficiary.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>United Microelectronics (UMC)</t>
+          <t>Quanta Computer</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>2303.TW</t>
+          <t>2382.TW</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Semis - Foundry</t>
+          <t>Data Center - AI Servers (ODM)</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="F36" s="9" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
@@ -1888,50 +1888,88 @@
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>1985-07</t>
+          <t>1999-01</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t>Mature/specialty foundry; 22/28nm; potential Intel collaboration optionality.</t>
+          <t>Top AI server ODM for US hyperscalers; cloud infrastructure leverage.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>SOUTH KOREA</t>
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>Wiwynn</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>6669.TW</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Data Center - AI Servers (ODM)</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>2019-03</t>
+        </is>
+      </c>
+      <c r="I37" s="10" t="inlineStr">
+        <is>
+          <t>Hyperscale-focused server pure-play (Wistron spin-off); Meta/Microsoft exposure.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>SK hynix</t>
+          <t>ASE Technology Holding</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>000660.KS</t>
+          <t>3711.TW</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>KRX</t>
+          <t>TWSE</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Semis - Memory (IDM)</t>
+          <t>Semis - OSAT</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="F38" s="9" t="n">
-        <v>800</v>
+        <v>25</v>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
@@ -1940,140 +1978,140 @@
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>1996-12</t>
+          <t>2018-04 (holding)</t>
         </is>
       </c>
       <c r="I38" s="10" t="inlineStr">
         <is>
-          <t>HBM leader into AI supercycle; primary NVIDIA HBM supplier; DRAM/NAND.</t>
+          <t>World's largest OSAT; advanced packaging/test capacity for AI chips.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>Samsung Electronics</t>
+          <t>United Microelectronics (UMC)</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>005930.KS</t>
+          <t>2303.TW</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Semis - Foundry</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>1985-07</t>
+        </is>
+      </c>
+      <c r="I39" s="10" t="inlineStr">
+        <is>
+          <t>Mature/specialty foundry; 22/28nm; potential Intel collaboration optionality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>SOUTH KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>SK hynix</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>000660.KS</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
           <t>KRX</t>
         </is>
       </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Semis - Memory/Foundry (IDM)</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Semis - Memory (IDM)</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
         <is>
           <t>South Korea</t>
         </is>
       </c>
-      <c r="F39" s="9" t="n">
-        <v>500</v>
-      </c>
-      <c r="G39" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H39" s="8" t="inlineStr">
-        <is>
-          <t>1975-06</t>
-        </is>
-      </c>
-      <c r="I39" s="10" t="inlineStr">
-        <is>
-          <t>DRAM/NAND/HBM + foundry + devices; HBM4 catch-up is the key AI catalyst.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>Hanmi Semiconductor</t>
-        </is>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>042700.KS</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>KRX</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Semis - Equipment (Packaging)</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>South Korea</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="G40" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H40" s="8" t="inlineStr">
-        <is>
-          <t>2005-07</t>
-        </is>
-      </c>
-      <c r="I40" s="10" t="inlineStr">
-        <is>
-          <t>TC bonders for HBM stacking (SK hynix/Micron supplier); pure-play AI memory equipment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>JAPAN</t>
+      <c r="F41" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>1996-12</t>
+        </is>
+      </c>
+      <c r="I41" s="10" t="inlineStr">
+        <is>
+          <t>HBM leader into AI supercycle; primary NVIDIA HBM supplier; DRAM/NAND.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>Tokyo Electron</t>
+          <t>Samsung Electronics</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>8035.T</t>
+          <t>005930.KS</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>TSE Prime</t>
+          <t>KRX</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>Semis - Equipment (WFE)</t>
+          <t>Semis - Memory/Foundry (IDM)</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="F42" s="9" t="n">
-        <v>150</v>
+        <v>500</v>
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
@@ -2082,43 +2120,43 @@
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>1980-10</t>
+          <t>1975-06</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr">
         <is>
-          <t>Top-tier WFE (coater/developer near-monopoly, etch, deposition); Japan flagship.</t>
+          <t>DRAM/NAND/HBM + foundry + devices; HBM4 catch-up is the key AI catalyst.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>Advantest</t>
+          <t>Hanmi Semiconductor</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>6857.T</t>
+          <t>042700.KS</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>TSE Prime</t>
+          <t>KRX</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Semis - Equipment (Test)</t>
+          <t>Semis - Equipment (Packaging)</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="F43" s="9" t="n">
-        <v>150</v>
+        <v>9</v>
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
@@ -2127,69 +2165,31 @@
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>1983-09</t>
+          <t>2005-07</t>
         </is>
       </c>
       <c r="I43" s="10" t="inlineStr">
         <is>
-          <t>Dominant SoC/memory tester; every AI accelerator and HBM stack needs test time.</t>
+          <t>TC bonders for HBM stacking (SK hynix/Micron supplier); pure-play AI memory equipment.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>Disco Corporation</t>
-        </is>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>6146.T</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>TSE Prime</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Semis - Equipment (Packaging)</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="G44" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H44" s="8" t="inlineStr">
-        <is>
-          <t>1989-11</t>
-        </is>
-      </c>
-      <c r="I44" s="10" t="inlineStr">
-        <is>
-          <t>Dicing/grinding near-monopoly; HBM wafer thinning; advanced packaging leverage.</t>
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>JAPAN</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Fujikura</t>
+          <t>Tokyo Electron</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>5803.T</t>
+          <t>8035.T</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Data Center - Optical Connectivity</t>
+          <t>Semis - Equipment (WFE)</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -2208,7 +2208,7 @@
         </is>
       </c>
       <c r="F45" s="9" t="n">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
@@ -2217,69 +2217,69 @@
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>1949 (TSE)</t>
+          <t>1980-10</t>
         </is>
       </c>
       <c r="I45" s="10" t="inlineStr">
         <is>
-          <t>Optical fiber/cable and high-density interconnect for AI datacenters; top TOPIX performer.</t>
+          <t>Top-tier WFE (coater/developer near-monopoly, etch, deposition); Japan flagship.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>Kioxia Holdings</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>285A.T</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>Advantest</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>TSE Prime</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Semis - Memory (NAND)</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Semis - Equipment (Test)</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="F46" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H46" s="5" t="inlineStr">
-        <is>
-          <t>2024-12</t>
-        </is>
-      </c>
-      <c r="I46" s="7" t="inlineStr">
-        <is>
-          <t>NAND flash pure-play (ex-Toshiba Memory); recent Tokyo IPO; AI storage demand.</t>
+      <c r="F46" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>1983-09</t>
+        </is>
+      </c>
+      <c r="I46" s="10" t="inlineStr">
+        <is>
+          <t>Dominant SoC/memory tester; every AI accelerator and HBM stack needs test time.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>Lasertec</t>
+          <t>Disco Corporation</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>6920.T</t>
+          <t>6146.T</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>Semis - Equipment (Inspection)</t>
+          <t>Semis - Equipment (Packaging)</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -2298,7 +2298,7 @@
         </is>
       </c>
       <c r="F47" s="9" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
@@ -2307,24 +2307,24 @@
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>1990-08</t>
+          <t>1989-11</t>
         </is>
       </c>
       <c r="I47" s="10" t="inlineStr">
         <is>
-          <t>Monopoly in EUV mask/blank inspection; leading-edge logic capex proxy.</t>
+          <t>Dicing/grinding near-monopoly; HBM wafer thinning; advanced packaging leverage.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>Ibiden</t>
+          <t>Fujikura</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>4062.T</t>
+          <t>5803.T</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>Semis - Substrates</t>
+          <t>Data Center - Optical Connectivity</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -2343,7 +2343,7 @@
         </is>
       </c>
       <c r="F48" s="9" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
@@ -2352,50 +2352,88 @@
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>1960s</t>
+          <t>1949 (TSE)</t>
         </is>
       </c>
       <c r="I48" s="10" t="inlineStr">
         <is>
-          <t>ABF package substrates for AI GPUs (NVIDIA supplier); capacity expansion cycle.</t>
+          <t>Optical fiber/cable and high-density interconnect for AI datacenters; top TOPIX performer.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>SINGAPORE</t>
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kioxia Holdings</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>285A.T</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>TSE Prime</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Semis - Memory (NAND)</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>NAND flash pure-play (ex-Toshiba Memory); recent Tokyo IPO; AI storage demand.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>Keppel DC REIT</t>
+          <t>Lasertec</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>AJBU.SI</t>
+          <t>6920.T</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>SGX</t>
+          <t>TSE Prime</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>Data Center - REIT</t>
+          <t>Semis - Equipment (Inspection)</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F50" s="9" t="n">
-        <v>4.3</v>
+        <v>20</v>
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
@@ -2404,121 +2442,271 @@
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t>2014-12</t>
+          <t>1990-08</t>
         </is>
       </c>
       <c r="I50" s="10" t="inlineStr">
         <is>
-          <t>Asia's first pure-play datacenter REIT; ~S$5B AUM, 20+ assets across 10 countries.</t>
+          <t>Monopoly in EUV mask/blank inspection; leading-edge logic capex proxy.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>NTT DC REIT</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>NTDU.SI</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>SGX</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Data Center - REIT</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H51" s="5" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="I51" s="7" t="inlineStr">
-        <is>
-          <t>Largest SGX REIT IPO in a decade (US$773M raise); NTT-sponsored global datacenter portfolio.</t>
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Ibiden</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>4062.T</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>TSE Prime</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Semis - Substrates</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>1960s</t>
+        </is>
+      </c>
+      <c r="I51" s="10" t="inlineStr">
+        <is>
+          <t>ABF package substrates for AI GPUs (NVIDIA supplier); capacity expansion cycle.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>MALAYSIA</t>
+          <t>SINGAPORE</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
+          <t>Keppel DC REIT</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>AJBU.SI</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>SGX</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Data Center - REIT</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>2014-12</t>
+        </is>
+      </c>
+      <c r="I53" s="10" t="inlineStr">
+        <is>
+          <t>Asia's first pure-play datacenter REIT; ~S$5B AUM, 20+ assets across 10 countries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>NTT DC REIT</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>NTDU.SI</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>SGX</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Data Center - REIT</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>Largest SGX REIT IPO in a decade (US$773M raise); NTT-sponsored global datacenter portfolio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>MALAYSIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
           <t>YTL Power International</t>
         </is>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>6742.KL</t>
         </is>
       </c>
-      <c r="C53" s="8" t="inlineStr">
+      <c r="C56" s="8" t="inlineStr">
         <is>
           <t>Bursa Malaysia</t>
         </is>
       </c>
-      <c r="D53" s="8" t="inlineStr">
+      <c r="D56" s="8" t="inlineStr">
         <is>
           <t>Data Center - Power/AI Campus</t>
         </is>
       </c>
-      <c r="E53" s="8" t="inlineStr">
+      <c r="E56" s="8" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="F53" s="9" t="n">
+      <c r="F56" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="G53" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H53" s="8" t="inlineStr">
+      <c r="G56" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H56" s="8" t="inlineStr">
         <is>
           <t>1997 (listed)</t>
         </is>
       </c>
-      <c r="I53" s="10" t="inlineStr">
+      <c r="I56" s="10" t="inlineStr">
         <is>
           <t>Utility building Johor AI datacenter campus (NVIDIA GPU cloud partnership); power + DC play.</t>
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>US ADR (CHINA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>VNET Group (21Vianet)</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>VNET</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Nasdaq (China ADR)</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Data Center - Colocation</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>US ADR (China)</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G58" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H58" s="8" t="inlineStr">
+        <is>
+          <t>2011-04</t>
+        </is>
+      </c>
+      <c r="I58" s="10" t="inlineStr">
+        <is>
+          <t>Carrier-neutral IDC in China; wholesale (Hyperscale 2.0) growth + retail; REIT/asset monetization optionality.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A52:I52"/>
-    <mergeCell ref="A41:I41"/>
-    <mergeCell ref="A49:I49"/>
-    <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A57:I57"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A37:I37"/>
-    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A55:I55"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2530,7 +2718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2568,10 +2756,10 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C2" s="12" t="n">
-        <v>677</v>
+        <v>899.3</v>
       </c>
       <c r="D2" s="12" t="n">
         <v>3</v>
@@ -2674,76 +2862,76 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>US ADR (China)</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n">
-        <v>42</v>
-      </c>
-      <c r="C9" s="13" t="n">
-        <v>4028.2</v>
-      </c>
-      <c r="D9" s="13" t="n">
+      <c r="B10" s="13" t="n">
+        <v>46</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>4252.9</v>
+      </c>
+      <c r="D10" s="13" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-    </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>By Subsector</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t># Names</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Agg. Approx. Mkt Cap ($B)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t># Recent IPOs</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Data Center - AI Servers (ODM)</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="C12" s="12" t="n">
-        <v>170</v>
-      </c>
-      <c r="D12" s="12" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>Data Center - Colocation</t>
+          <t>Data Center - AI Servers (ODM)</t>
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>9.4</v>
+        <v>170</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>0</v>
@@ -2752,14 +2940,14 @@
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>Data Center - IDC/Cloud</t>
+          <t>Data Center - Cloud/AI Compute</t>
         </is>
       </c>
       <c r="B14" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>4</v>
+        <v>2.3</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>0</v>
@@ -2768,14 +2956,14 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Data Center - Optical Connectivity</t>
+          <t>Data Center - Colocation</t>
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>25</v>
+        <v>11.8</v>
       </c>
       <c r="D15" s="12" t="n">
         <v>0</v>
@@ -2784,14 +2972,14 @@
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>Data Center - Power/AI Campus</t>
+          <t>Data Center - IDC/Cloud</t>
         </is>
       </c>
       <c r="B16" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D16" s="12" t="n">
         <v>0</v>
@@ -2800,14 +2988,14 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Data Center - Power/Cooling</t>
+          <t>Data Center - Optical Connectivity</t>
         </is>
       </c>
       <c r="B17" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>0</v>
@@ -2816,30 +3004,30 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>Data Center - REIT</t>
+          <t>Data Center - Optical Modules</t>
         </is>
       </c>
       <c r="B18" s="12" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="12" t="n">
-        <v>5.3</v>
+        <v>220</v>
       </c>
       <c r="D18" s="12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>Data Center - Wholesale IDC</t>
+          <t>Data Center - Power/AI Campus</t>
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>0</v>
@@ -2848,14 +3036,14 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>Semis - AI Accelerators</t>
+          <t>Data Center - Power/Cooling</t>
         </is>
       </c>
       <c r="B20" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="12" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>0</v>
@@ -2864,30 +3052,30 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Semis - Auto AI SoC</t>
+          <t>Data Center - REIT</t>
         </is>
       </c>
       <c r="B21" s="12" t="n">
         <v>2</v>
       </c>
       <c r="C21" s="12" t="n">
-        <v>10.5</v>
+        <v>5.3</v>
       </c>
       <c r="D21" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>Semis - CPU/DCU</t>
+          <t>Data Center - Wholesale IDC</t>
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" s="12" t="n">
-        <v>95</v>
+        <v>13</v>
       </c>
       <c r="D22" s="12" t="n">
         <v>0</v>
@@ -2896,14 +3084,14 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>Semis - Equipment (Inspection)</t>
+          <t>Semis - AI Accelerators</t>
         </is>
       </c>
       <c r="B23" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="12" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="D23" s="12" t="n">
         <v>0</v>
@@ -2912,30 +3100,30 @@
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>Semis - Equipment (Packaging)</t>
+          <t>Semis - Auto AI SoC</t>
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C24" s="12" t="n">
-        <v>50</v>
+        <v>10.5</v>
       </c>
       <c r="D24" s="12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>Semis - Equipment (Test)</t>
+          <t>Semis - CPU/DCU</t>
         </is>
       </c>
       <c r="B25" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="12" t="n">
-        <v>150</v>
+        <v>95</v>
       </c>
       <c r="D25" s="12" t="n">
         <v>0</v>
@@ -2944,14 +3132,14 @@
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Semis - Equipment (WFE)</t>
+          <t>Semis - Equipment (Inspection)</t>
         </is>
       </c>
       <c r="B26" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C26" s="12" t="n">
-        <v>235</v>
+        <v>20</v>
       </c>
       <c r="D26" s="12" t="n">
         <v>0</v>
@@ -2960,14 +3148,14 @@
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>Semis - Fabless (SoC)</t>
+          <t>Semis - Equipment (Packaging)</t>
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C27" s="12" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="D27" s="12" t="n">
         <v>0</v>
@@ -2976,14 +3164,14 @@
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>Semis - Foundry</t>
+          <t>Semis - Equipment (Test)</t>
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C28" s="12" t="n">
-        <v>1348</v>
+        <v>150</v>
       </c>
       <c r="D28" s="12" t="n">
         <v>0</v>
@@ -2992,46 +3180,46 @@
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>Semis - GPU</t>
+          <t>Semis - Equipment (WFE)</t>
         </is>
       </c>
       <c r="B29" s="12" t="n">
         <v>3</v>
       </c>
       <c r="C29" s="12" t="n">
-        <v>88</v>
+        <v>235</v>
       </c>
       <c r="D29" s="12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>Semis - Memory (DRAM)</t>
+          <t>Semis - Fabless (SoC)</t>
         </is>
       </c>
       <c r="B30" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="12" t="n">
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="D30" s="12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Semis - Memory (IDM)</t>
+          <t>Semis - Foundry</t>
         </is>
       </c>
       <c r="B31" s="12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C31" s="12" t="n">
-        <v>800</v>
+        <v>1348</v>
       </c>
       <c r="D31" s="12" t="n">
         <v>0</v>
@@ -3040,46 +3228,46 @@
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>Semis - Memory (NAND)</t>
+          <t>Semis - GPU</t>
         </is>
       </c>
       <c r="B32" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C32" s="12" t="n">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="D32" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>Semis - Memory (NOR/NAND/DRAM)</t>
+          <t>Semis - Memory (DRAM)</t>
         </is>
       </c>
       <c r="B33" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="12" t="n">
-        <v>12</v>
+        <v>150</v>
       </c>
       <c r="D33" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>Semis - Memory Interface</t>
+          <t>Semis - Memory (IDM)</t>
         </is>
       </c>
       <c r="B34" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="12" t="n">
-        <v>15</v>
+        <v>800</v>
       </c>
       <c r="D34" s="12" t="n">
         <v>0</v>
@@ -3088,30 +3276,30 @@
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>Semis - Memory/Foundry (IDM)</t>
+          <t>Semis - Memory (NAND)</t>
         </is>
       </c>
       <c r="B35" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="12" t="n">
-        <v>500</v>
+        <v>20</v>
       </c>
       <c r="D35" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>Semis - OSAT</t>
+          <t>Semis - Memory (NOR/NAND/DRAM)</t>
         </is>
       </c>
       <c r="B36" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="12" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D36" s="12" t="n">
         <v>0</v>
@@ -3120,32 +3308,80 @@
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>Semis - Power (GaN)</t>
+          <t>Semis - Memory Interface</t>
         </is>
       </c>
       <c r="B37" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="12" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D37" s="12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t>Semis - Substrates</t>
+          <t>Semis - Memory/Foundry (IDM)</t>
         </is>
       </c>
       <c r="B38" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="D38" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Semis - OSAT</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D39" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>Semis - Power (GaN)</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D40" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Semis - Substrates</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="D38" s="12" t="n">
+      <c r="D41" s="12" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>